<commit_message>
🚀 Matriz procesada (Checkpoint de seguridad) por GitHub Actions
</commit_message>
<xml_diff>
--- a/outputs/matriz_procesada.xlsx
+++ b/outputs/matriz_procesada.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:ZZ5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14.42578125" customWidth="1" min="1" max="1"/>
@@ -512,6 +512,11 @@
         </is>
       </c>
       <c r="F1" s="4" t="n"/>
+      <c r="ZZ1" t="inlineStr">
+        <is>
+          <t>Trigger: 1786133639.465325</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="C2" s="4" t="inlineStr">

</xml_diff>